<commit_message>
feat(socios): separar calle, numero, ciudad y provincia en las direcciones
Pedido del cliente: la direccion venia toda junta en un campo. Ahora
`direccion` y `direccion_fiscal` son solo la calle, y se agregan numero
(en las dos) mas ciudad y provincia para la fiscal, que antes no las
tenia separadas.

Cubre alta de socio, ficha (Generales y Datos Impositivos), carga masiva
por Excel (columna `numero` nueva + plantilla regenerada) y el buscador
de socios de Ventas.

Lo que va a ARCA no cambia: `armarDomicilio` vuelve a unir las partes en
una linea antes de mandar el comprobante.

Mig 0143 con backfill: parte los valores existentes por coma y por el
numero al final. Probado en seco contra los 15 socios cargados antes de
aplicarlo; las direcciones sin numero quedan enteras en la calle.
</commit_message>
<xml_diff>
--- a/public/templates/socios.xlsx
+++ b/public/templates/socios.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>nombre *</t>
   </si>
@@ -29,6 +29,9 @@
     <t>direccion</t>
   </si>
   <si>
+    <t>numero</t>
+  </si>
+  <si>
     <t>tipo_documento</t>
   </si>
   <si>
@@ -53,7 +56,10 @@
     <t>Teléfono (opcional)</t>
   </si>
   <si>
-    <t>Dirección (opcional)</t>
+    <t>Calle, sin el número (opcional)</t>
+  </si>
+  <si>
+    <t>Número de la calle (opcional)</t>
   </si>
   <si>
     <t>DNI, CUIT o CUIL</t>
@@ -80,7 +86,10 @@
     <t>11-1234-5678</t>
   </si>
   <si>
-    <t>Av. Costanera 123</t>
+    <t>Av. Costanera</t>
+  </si>
+  <si>
+    <t>123</t>
   </si>
   <si>
     <t>DNI</t>
@@ -587,20 +596,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,66 +638,75 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -697,8 +716,9 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="4"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -708,8 +728,9 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="4"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -719,8 +740,9 @@
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" s="4"/>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -730,8 +752,9 @@
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="4"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -741,8 +764,9 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="4"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -752,8 +776,9 @@
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="4"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -763,8 +788,9 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -774,8 +800,9 @@
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -785,8 +812,9 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -796,8 +824,9 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -807,8 +836,9 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -818,8 +848,9 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="4"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -829,8 +860,9 @@
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" s="4"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -840,8 +872,9 @@
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -851,8 +884,9 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -862,8 +896,9 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" s="4"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -873,8 +908,9 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -884,8 +920,9 @@
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -895,8 +932,9 @@
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -906,8 +944,9 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="4"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -917,8 +956,9 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -928,8 +968,9 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -939,8 +980,9 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -950,8 +992,9 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -961,8 +1004,9 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -972,8 +1016,9 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -983,8 +1028,9 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" s="4"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -994,8 +1040,9 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" s="4"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1005,8 +1052,9 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" s="4"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1016,8 +1064,9 @@
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="4"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1027,8 +1076,9 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="4"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -1038,8 +1088,9 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
-    </row>
-    <row r="36" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1049,8 +1100,9 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
-    </row>
-    <row r="37" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="4"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -1060,8 +1112,9 @@
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
-    </row>
-    <row r="38" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" s="4"/>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -1071,8 +1124,9 @@
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
-    </row>
-    <row r="39" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -1082,8 +1136,9 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -1093,8 +1148,9 @@
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
-    </row>
-    <row r="41" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" s="4"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -1104,8 +1160,9 @@
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
-    </row>
-    <row r="42" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" s="4"/>
+    </row>
+    <row r="42" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -1115,8 +1172,9 @@
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-    </row>
-    <row r="43" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" s="4"/>
+    </row>
+    <row r="43" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -1126,8 +1184,9 @@
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
-    </row>
-    <row r="44" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1137,8 +1196,9 @@
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
-    </row>
-    <row r="45" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" s="4"/>
+    </row>
+    <row r="45" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -1148,8 +1208,9 @@
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
-    </row>
-    <row r="46" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" s="4"/>
+    </row>
+    <row r="46" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -1159,8 +1220,9 @@
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" s="4"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -1170,8 +1232,9 @@
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
-    </row>
-    <row r="48" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" s="4"/>
+    </row>
+    <row r="48" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -1181,8 +1244,9 @@
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
-    </row>
-    <row r="49" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -1192,8 +1256,9 @@
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
-    </row>
-    <row r="50" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1203,6 +1268,7 @@
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1220,82 +1286,82 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>